<commit_message>
función para ejecutar varias instancias con varios solvers
</commit_message>
<xml_diff>
--- a/data/inst_1.xlsx
+++ b/data/inst_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marta_sierra\PycharmProjects\Flexible-vrp\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\TFG\Flexible\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BDA322-FEB2-4383-802F-5980CCF15D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9B5CC17-FFAF-458D-A3B2-198370E5FE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3960" yWindow="1470" windowWidth="15375" windowHeight="12150" xr2:uid="{5A598FCB-B967-4DAF-9410-AD9F1FA49DAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5A598FCB-B967-4DAF-9410-AD9F1FA49DAC}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="3" r:id="rId1"/>
@@ -25,12 +25,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>origin</t>
   </si>
@@ -41,25 +52,7 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>F1</t>
-  </si>
-  <si>
     <t>T1</t>
-  </si>
-  <si>
-    <t>T3</t>
-  </si>
-  <si>
-    <t>T4</t>
-  </si>
-  <si>
-    <t>T5</t>
-  </si>
-  <si>
-    <t>F2</t>
-  </si>
-  <si>
-    <t>F3</t>
   </si>
   <si>
     <t>T2</t>
@@ -203,8 +196,8 @@
       <sheetName val="comp_quantity_inst1"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1">
         <row r="2">
           <cell r="C2">
             <v>5</v>
@@ -486,16 +479,16 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="2" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -533,7 +526,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -639,7 +632,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -781,7 +774,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -797,15 +790,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>22</v>
@@ -813,7 +806,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
@@ -821,7 +814,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -829,7 +822,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0.5</v>
@@ -837,7 +830,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2">
         <v>480</v>
@@ -845,7 +838,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>600</v>
@@ -853,7 +846,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -861,7 +854,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B9">
         <v>600</v>
@@ -869,7 +862,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <v>120</v>
@@ -877,7 +870,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1">
         <f>AVERAGE([1]trip_duration!C2:C57)</f>
@@ -886,23 +879,24 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B12" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B13">
-        <v>41</v>
+        <f>SUM(comp_quantity_inst1!C2:C3)</f>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <v>108</v>
@@ -910,10 +904,10 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -923,26 +917,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2A54DE7-45BC-48AF-A573-13FFF226C261}">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -953,603 +947,9 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" t="s">
-        <v>3</v>
-      </c>
-      <c r="C20">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>5</v>
-      </c>
-      <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>6</v>
-      </c>
-      <c r="B23" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>6</v>
-      </c>
-      <c r="B24" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>6</v>
-      </c>
-      <c r="B27" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>6</v>
-      </c>
-      <c r="B28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>7</v>
-      </c>
-      <c r="B31" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" t="s">
-        <v>5</v>
-      </c>
-      <c r="C32">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>7</v>
-      </c>
-      <c r="B33" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>7</v>
-      </c>
-      <c r="B34" t="s">
-        <v>3</v>
-      </c>
-      <c r="C34">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>3</v>
-      </c>
-      <c r="B37" t="s">
-        <v>4</v>
-      </c>
-      <c r="C37">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>3</v>
-      </c>
-      <c r="B38" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>3</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>3</v>
-      </c>
-      <c r="B40" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>3</v>
-      </c>
-      <c r="B41" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>3</v>
-      </c>
-      <c r="B42" t="s">
-        <v>8</v>
-      </c>
-      <c r="C42">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>3</v>
-      </c>
-      <c r="B43" t="s">
-        <v>9</v>
-      </c>
-      <c r="C43">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>8</v>
-      </c>
-      <c r="B44" t="s">
-        <v>4</v>
-      </c>
-      <c r="C44">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>8</v>
-      </c>
-      <c r="B45" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>8</v>
-      </c>
-      <c r="B46" t="s">
-        <v>5</v>
-      </c>
-      <c r="C46">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>8</v>
-      </c>
-      <c r="B47" t="s">
-        <v>6</v>
-      </c>
-      <c r="C47">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>8</v>
-      </c>
-      <c r="B48" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" t="s">
-        <v>3</v>
-      </c>
-      <c r="C49">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>8</v>
-      </c>
-      <c r="B50" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>9</v>
-      </c>
-      <c r="B51" t="s">
-        <v>4</v>
-      </c>
-      <c r="C51">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>9</v>
-      </c>
-      <c r="B52" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>9</v>
-      </c>
-      <c r="B53" t="s">
-        <v>5</v>
-      </c>
-      <c r="C53">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>9</v>
-      </c>
-      <c r="B54" t="s">
-        <v>6</v>
-      </c>
-      <c r="C54">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>9</v>
-      </c>
-      <c r="B55" t="s">
-        <v>7</v>
-      </c>
-      <c r="C55">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>9</v>
-      </c>
-      <c r="B56" t="s">
-        <v>3</v>
-      </c>
-      <c r="C56">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>9</v>
-      </c>
-      <c r="B57" t="s">
-        <v>8</v>
-      </c>
-      <c r="C57">
         <v>5</v>
       </c>
     </row>
@@ -1574,15 +974,15 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
       </c>
       <c r="C2">
         <v>12</v>
@@ -1593,10 +993,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>19</v>
@@ -1607,10 +1007,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
       </c>
       <c r="C4">
         <v>50</v>
@@ -1621,10 +1021,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5">
         <v>58</v>

</xml_diff>